<commit_message>
Made instructions in code clearer
</commit_message>
<xml_diff>
--- a/Notes/CPU_Instruction_Set.xlsx
+++ b/Notes/CPU_Instruction_Set.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Reyansh\BOLT-16_CPU\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Reyansh\BOLT-16_CPU\Notes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3EBC09E-7D0A-4692-B913-417034C38621}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A30F155-9430-49FF-A0C7-2B19BABD3997}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{25FB4FC9-3870-4051-8B39-19FFBC5F0F37}"/>
   </bookViews>
@@ -660,7 +660,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.88671875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="93.21875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="17.77734375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="11.109375" bestFit="1" customWidth="1"/>

</xml_diff>